<commit_message>
Atualiza medicao e funcionarios
</commit_message>
<xml_diff>
--- a/doc/docs/medicao.xlsx
+++ b/doc/docs/medicao.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr hidePivotFieldList="1"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <workbookPr hidePivotFieldList="1" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micro\Desktop\moderno\dashboard-obras\github\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A23AC0DF-D76F-4289-81EA-2D7C3B096339}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17DF90F4-BCD8-4329-9567-FC16760B6984}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-45" windowWidth="29040" windowHeight="15720" xr2:uid="{C4B49546-303A-44FC-A2B7-442D4305AD02}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C4B49546-303A-44FC-A2B7-442D4305AD02}"/>
   </bookViews>
   <sheets>
     <sheet name="medição" sheetId="5" r:id="rId1"/>
@@ -679,15 +679,16 @@
         <v>13600196.199999999</v>
       </c>
       <c r="C10" s="5">
-        <v>2630306.9</v>
+        <f>2630306.9/2</f>
+        <v>1315153.45</v>
       </c>
       <c r="E10" s="1">
         <f t="shared" si="0"/>
-        <v>10969889.299999999</v>
+        <v>12285042.75</v>
       </c>
       <c r="F10" s="6">
         <f>C10/B10</f>
-        <v>0.19340212900752124</v>
+        <v>9.670106450376062E-2</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
@@ -737,13 +738,13 @@
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="J16" s="2">
         <f>SUM(C2:C11)</f>
-        <v>20779424.5068</v>
+        <v>19464271.0568</v>
       </c>
     </row>
     <row r="17" spans="10:10" x14ac:dyDescent="0.3">
       <c r="J17" s="2">
         <f>J15-J16</f>
-        <v>119338560.44320002</v>
+        <v>120653713.89320001</v>
       </c>
     </row>
     <row r="20" spans="10:10" x14ac:dyDescent="0.3">
@@ -1024,6 +1025,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <Users xmlns="84c92d79-736b-434d-a6de-4a5b6bb0f72c">
@@ -1042,15 +1052,6 @@
     <_Flow_SignoffStatus xmlns="84c92d79-736b-434d-a6de-4a5b6bb0f72c" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1074,6 +1075,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D6D777F3-47C0-461C-AB58-3D988F0D0DFE}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8FE54049-832F-4559-A380-4B2190B687C3}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -1083,12 +1092,4 @@
     <ds:schemaRef ds:uri="de022bf3-4aff-41f6-a825-e7793343a5a1"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D6D777F3-47C0-461C-AB58-3D988F0D0DFE}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>